<commit_message>
Hemanth author sheet update
</commit_message>
<xml_diff>
--- a/author.xlsx
+++ b/author.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11008"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A02844-8142-46B4-88F1-ACABB30F9D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{32A02844-8142-46B4-88F1-ACABB30F9D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E42F5CFD-EB11-B34B-95DB-9CB66E653DD3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="4" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="71">
   <si>
     <t>Short Description</t>
   </si>
@@ -37,18 +37,12 @@
     <t>Date of birth:</t>
   </si>
   <si>
-    <t>&lt;01.01.2000&gt;</t>
-  </si>
-  <si>
     <t>Address:</t>
   </si>
   <si>
     <t>Street home:</t>
   </si>
   <si>
-    <t>&lt;Steinweg 15&gt;</t>
-  </si>
-  <si>
     <t>City home:</t>
   </si>
   <si>
@@ -58,12 +52,6 @@
     <t>Company name/Department:</t>
   </si>
   <si>
-    <t>&lt;Hochschule Emden/Leer&gt; or &lt; VW Wolfsburg&gt; or &lt;...&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Fachbereich Technik&gt;  or &lt;Strak&gt; or &lt;...&gt;</t>
-  </si>
-  <si>
     <t>Street Workplace:</t>
   </si>
   <si>
@@ -76,24 +64,12 @@
     <t>Supervisor workplace:</t>
   </si>
   <si>
-    <t>&lt;Einstein, Albert&gt;</t>
-  </si>
-  <si>
-    <t>&lt;00494921 807-1001&gt;</t>
-  </si>
-  <si>
     <t>Email:</t>
   </si>
   <si>
-    <t>&lt;albert.einstein@hs-emden-leer.de&gt;</t>
-  </si>
-  <si>
     <t>Second examiner:</t>
   </si>
   <si>
-    <t>&lt;Prof. Dr. Carla Columna&gt;</t>
-  </si>
-  <si>
     <t>Outstanding examinations:</t>
   </si>
   <si>
@@ -145,15 +121,9 @@
     <t xml:space="preserve">Study: </t>
   </si>
   <si>
-    <t>&lt;04921 807 1429&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">Workplace: </t>
   </si>
   <si>
-    <t>&lt;04921 807 1428&gt;</t>
-  </si>
-  <si>
     <t>Name, Surname</t>
   </si>
   <si>
@@ -248,6 +218,24 @@
   </si>
   <si>
     <t>&lt;0157 333 47 662&gt;</t>
+  </si>
+  <si>
+    <t>Hemanth-Jp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hemanth.jadiswami.prabhakaran@stud.hs-emden-leer.de </t>
+  </si>
+  <si>
+    <t>hemanthjp139@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &lt;10&gt;</t>
+  </si>
+  <si>
+    <t>&lt;06.01.1996&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Graf-Johann-Straße 16 Port Arthur&gt;</t>
   </si>
 </sst>
 </file>
@@ -638,18 +626,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N7"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="11.5703125" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" customWidth="1"/>
+    <col min="1" max="2" width="11.5" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="5" width="11.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="33.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:14" ht="34" x14ac:dyDescent="0.4">
       <c r="A1" s="7"/>
       <c r="B1" s="6"/>
       <c r="C1" s="11" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
@@ -663,26 +651,26 @@
       <c r="M1" s="11"/>
       <c r="N1" s="11"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -701,73 +689,73 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A3:F50"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.33203125" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="3" max="3" width="33.1640625" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="43" customWidth="1"/>
-    <col min="6" max="6" width="24.42578125" customWidth="1"/>
+    <col min="6" max="6" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C5" s="8">
         <v>7026116</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C6" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -775,200 +763,200 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1">
         <v>45595</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1">
         <v>45688</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="B22" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B22" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="B23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="B28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B25" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B38" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B28" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="B40" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B29" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="3"/>
-    </row>
-    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A37" s="5" t="s">
+      <c r="B50" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A44" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B45" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B46" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B47" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B50" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -991,70 +979,70 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:F50"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C5" s="2">
         <v>7025671</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C6" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1062,200 +1050,200 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1">
         <v>45595</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1">
         <v>45688</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="B22" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B22" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="B23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B23" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="B25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B25" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B38" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B28" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="B40" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B29" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="3"/>
-    </row>
-    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A37" s="5" t="s">
+      <c r="B50" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A44" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B45" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B46" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B47" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B50" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1277,269 +1265,272 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A3:F50"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2">
-        <v>1234567</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>7026000</v>
+      </c>
+      <c r="D5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C6" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B10">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1">
-        <v>45351</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45595</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1">
-        <v>45594</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45688</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="B22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="B28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B38" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B28" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+      <c r="B40" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="3"/>
+    </row>
+    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B29" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B45" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="3"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B34" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="3"/>
-    </row>
-    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A37" s="5" t="s">
+      <c r="B50" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B39" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B40" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-    </row>
-    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="A44" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B45" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B46" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B47" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B50" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manual update and introduction
</commit_message>
<xml_diff>
--- a/author.xlsx
+++ b/author.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10112"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49CF5DD5-A491-401F-930E-21D54EECFD68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925B31AB-98C7-594A-9BB6-CDC32538E85C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="680" windowWidth="23260" windowHeight="12580" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="4" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="65">
   <si>
     <t>Short Description</t>
   </si>
@@ -212,21 +212,6 @@
   </si>
   <si>
     <t>Masters in Business Intelligence and Data Analytics</t>
-  </si>
-  <si>
-    <t>Vedant</t>
-  </si>
-  <si>
-    <t>Purohit</t>
-  </si>
-  <si>
-    <t>Ved-Purohit22</t>
-  </si>
-  <si>
-    <t>vedant.ramkrishna.purohit@stud.hs-emden-leer.de</t>
-  </si>
-  <si>
-    <t>ved.purohit22@gmail.com</t>
   </si>
   <si>
     <t>22.12.1999</t>
@@ -612,36 +597,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="63.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.6" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:3" ht="34" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>50</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -659,21 +644,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A3:F50"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="47.33203125" customWidth="1"/>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.109375" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.1640625" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -693,7 +678,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -713,10 +698,10 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C6" s="1"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -724,10 +709,10 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>2</v>
       </c>
@@ -735,10 +720,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
@@ -746,7 +731,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -754,10 +739,10 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -765,7 +750,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
@@ -773,13 +758,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>3</v>
       </c>
@@ -787,16 +772,16 @@
         <v>36534</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
@@ -804,7 +789,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>6</v>
       </c>
@@ -812,10 +797,10 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>7</v>
       </c>
@@ -823,17 +808,17 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>8</v>
       </c>
@@ -841,7 +826,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>9</v>
       </c>
@@ -849,19 +834,19 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>28</v>
       </c>
@@ -869,29 +854,29 @@
         <v>15510820227</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>31</v>
       </c>
@@ -899,7 +884,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>10</v>
       </c>
@@ -907,7 +892,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>14</v>
       </c>
@@ -915,25 +900,25 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>31</v>
       </c>
@@ -941,7 +926,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>10</v>
       </c>
@@ -949,7 +934,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>14</v>
       </c>
@@ -957,13 +942,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>18</v>
       </c>
@@ -990,21 +975,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:F50"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1024,7 +1009,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -1044,10 +1029,10 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C6" s="1"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -1055,10 +1040,10 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>2</v>
       </c>
@@ -1066,10 +1051,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
@@ -1077,7 +1062,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -1085,10 +1070,10 @@
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -1096,7 +1081,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
@@ -1104,13 +1089,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>3</v>
       </c>
@@ -1118,16 +1103,16 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
@@ -1135,7 +1120,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>6</v>
       </c>
@@ -1143,10 +1128,10 @@
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>7</v>
       </c>
@@ -1154,17 +1139,17 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>8</v>
       </c>
@@ -1172,7 +1157,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>9</v>
       </c>
@@ -1180,13 +1165,13 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>10</v>
       </c>
@@ -1194,35 +1179,35 @@
         <v>15510941084</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>31</v>
       </c>
@@ -1230,7 +1215,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>10</v>
       </c>
@@ -1238,7 +1223,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>14</v>
       </c>
@@ -1246,25 +1231,25 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>31</v>
       </c>
@@ -1272,7 +1257,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>10</v>
       </c>
@@ -1280,7 +1265,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>14</v>
       </c>
@@ -1288,13 +1273,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>18</v>
       </c>
@@ -1321,21 +1306,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A3:F50"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="43.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1355,30 +1340,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="1">
-        <v>7027292</v>
-      </c>
-      <c r="D5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E5" t="s">
-        <v>66</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C5" s="1"/>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C6" s="1"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -1386,7 +1355,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>2</v>
       </c>
@@ -1394,7 +1363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
@@ -1402,7 +1371,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -1410,7 +1379,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -1418,7 +1387,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
@@ -1426,28 +1395,28 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>6</v>
       </c>
@@ -1455,7 +1424,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>7</v>
       </c>
@@ -1463,17 +1432,17 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>8</v>
       </c>
@@ -1481,7 +1450,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>9</v>
       </c>
@@ -1489,35 +1458,35 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
     </row>
-    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>31</v>
       </c>
@@ -1525,7 +1494,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>10</v>
       </c>
@@ -1533,7 +1502,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>14</v>
       </c>
@@ -1541,21 +1510,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
     </row>
-    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>31</v>
       </c>
@@ -1563,7 +1532,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>10</v>
       </c>
@@ -1571,7 +1540,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>14</v>
       </c>
@@ -1579,13 +1548,13 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>18</v>
       </c>
@@ -1600,9 +1569,6 @@
       <formula1>"Technical Management, Business Intelligen ans Data Analytics,Maschinenbau,Indin,IBS,Maschinenbau und Design,Maschinenbau und Design im Praxisverbund,Engineering Physics,other"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="F5" r:id="rId1" xr:uid="{37BDC1F4-AC28-461A-83EA-E10A8AB698A1}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>